<commit_message>
docs+wizard: group AGC with App Gateway and clarify either/or ingress choice
- Checklist: renumber add-ons contiguously (enable_agc is now 11g, right after
  enable_app_gateway 11f; keda..cost_analysis shift to 11h..11p). Both ingress
  rows state 'choose this OR the other - not both'; fix 5h cross-ref to 11g.
- Wizard: clarify the two ingress prompt labels as mutually-exclusive options A/B.
</commit_message>
<xml_diff>
--- a/docs/assets/aks-landing-zone-checklist.xlsx
+++ b/docs/assets/aks-landing-zone-checklist.xlsx
@@ -1831,7 +1831,7 @@
       </c>
       <c r="C29" s="17" t="inlineStr">
         <is>
-          <t>App Gateway for Containers subnet (delegated, min /24). Used only when 11p = true.</t>
+          <t>App Gateway for Containers subnet (delegated, min /24). Used only when 11g = true.</t>
         </is>
       </c>
       <c r="D29" s="18" t="inlineStr">
@@ -2591,7 +2591,7 @@
       </c>
       <c r="C55" s="17" t="inlineStr">
         <is>
-          <t>Application Gateway + WAF in front of the cluster.</t>
+          <t>Application Gateway + WAF in front of the cluster. Classic L7 ingress. Choose this OR App Gateway for Containers (11g) — not both.</t>
         </is>
       </c>
       <c r="D55" s="18" t="inlineStr">
@@ -2615,7 +2615,7 @@
     <row r="56" ht="42" customHeight="1">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t>11p</t>
+          <t>11g</t>
         </is>
       </c>
       <c r="B56" s="9" t="inlineStr">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="C56" s="10" t="inlineStr">
         <is>
-          <t>Application Gateway for Containers (ALB). Provisions delegated subnet 5h and ALB Controller.</t>
+          <t>Application Gateway for Containers (ALB) — next-gen L7 ingress. Provisions delegated subnet 5h and ALB Controller. Choose this OR Application Gateway WAF (11f) — not both.</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
@@ -2649,7 +2649,7 @@
     <row r="57" ht="42" customHeight="1">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>11g</t>
+          <t>11h</t>
         </is>
       </c>
       <c r="B57" s="16" t="inlineStr">
@@ -2683,7 +2683,7 @@
     <row r="58" ht="42" customHeight="1">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t>11h</t>
+          <t>11i</t>
         </is>
       </c>
       <c r="B58" s="9" t="inlineStr">
@@ -2717,7 +2717,7 @@
     <row r="59" ht="42" customHeight="1">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>11i</t>
+          <t>11j</t>
         </is>
       </c>
       <c r="B59" s="16" t="inlineStr">
@@ -2751,7 +2751,7 @@
     <row r="60" ht="42" customHeight="1">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t>11j</t>
+          <t>11k</t>
         </is>
       </c>
       <c r="B60" s="9" t="inlineStr">
@@ -2785,7 +2785,7 @@
     <row r="61" ht="42" customHeight="1">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>11k</t>
+          <t>11l</t>
         </is>
       </c>
       <c r="B61" s="16" t="inlineStr">
@@ -2819,7 +2819,7 @@
     <row r="62" ht="42" customHeight="1">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t>11l</t>
+          <t>11m</t>
         </is>
       </c>
       <c r="B62" s="9" t="inlineStr">
@@ -2853,7 +2853,7 @@
     <row r="63" ht="42" customHeight="1">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>11m</t>
+          <t>11n</t>
         </is>
       </c>
       <c r="B63" s="16" t="inlineStr">
@@ -2887,7 +2887,7 @@
     <row r="64" ht="42" customHeight="1">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t>11n</t>
+          <t>11o</t>
         </is>
       </c>
       <c r="B64" s="9" t="inlineStr">
@@ -2921,7 +2921,7 @@
     <row r="65" ht="42" customHeight="1">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>11o</t>
+          <t>11p</t>
         </is>
       </c>
       <c r="B65" s="16" t="inlineStr">

</xml_diff>